<commit_message>
fix color of "FAIILED"
</commit_message>
<xml_diff>
--- a/playwright-test/test-case.xlsx
+++ b/playwright-test/test-case.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5C1E5C-E2FA-4C22-85FD-BAA50EA42227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{489A05FB-BC42-4615-B5F6-E38F2EADC729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="90">
   <si>
     <t>Test case</t>
   </si>
@@ -249,58 +249,58 @@
     <t>error-email</t>
   </si>
   <si>
+    <t>Báo lỗi bỏ trống password</t>
+  </si>
+  <si>
+    <t>error-password</t>
+  </si>
+  <si>
+    <t>Password cần ít nhất 6 kí tự</t>
+  </si>
+  <si>
+    <t>Nhập email sai định dạng</t>
+  </si>
+  <si>
+    <t>user@</t>
+  </si>
+  <si>
+    <t>Nhập mật khẩu hợp lệ</t>
+  </si>
+  <si>
+    <t>Báo lỗi định dạng email</t>
+  </si>
+  <si>
+    <t>Email không đúng định dạng</t>
+  </si>
+  <si>
+    <t>Nhập email tài khoản</t>
+  </si>
+  <si>
+    <t>admin@example.com</t>
+  </si>
+  <si>
+    <t>Nhập sai mật khẩu</t>
+  </si>
+  <si>
+    <t>WrongPass123</t>
+  </si>
+  <si>
+    <t>Báo lỗi sai thông tin đăng nhập</t>
+  </si>
+  <si>
+    <t>css</t>
+  </si>
+  <si>
+    <t>[data-sonner-toast]</t>
+  </si>
+  <si>
+    <t>/</t>
+  </si>
+  <si>
+    <t>Tài khoản hoặc mật khẩu không chính xác</t>
+  </si>
+  <si>
     <t>Email cần ít nhất 3 kí tự</t>
-  </si>
-  <si>
-    <t>Báo lỗi bỏ trống password</t>
-  </si>
-  <si>
-    <t>error-password</t>
-  </si>
-  <si>
-    <t>Password cần ít nhất 6 kí tự</t>
-  </si>
-  <si>
-    <t>Nhập email sai định dạng</t>
-  </si>
-  <si>
-    <t>user@</t>
-  </si>
-  <si>
-    <t>Nhập mật khẩu hợp lệ</t>
-  </si>
-  <si>
-    <t>Báo lỗi định dạng email</t>
-  </si>
-  <si>
-    <t>Email không đúng định dạng</t>
-  </si>
-  <si>
-    <t>Nhập email tài khoản</t>
-  </si>
-  <si>
-    <t>admin@example.com</t>
-  </si>
-  <si>
-    <t>Nhập sai mật khẩu</t>
-  </si>
-  <si>
-    <t>WrongPass123</t>
-  </si>
-  <si>
-    <t>Báo lỗi sai thông tin đăng nhập</t>
-  </si>
-  <si>
-    <t>css</t>
-  </si>
-  <si>
-    <t>[data-sonner-toast]</t>
-  </si>
-  <si>
-    <t>Tài khoản hoặc mật khẩu không chính xác</t>
-  </si>
-  <si>
-    <t>/dashboard</t>
   </si>
 </sst>
 </file>
@@ -1136,7 +1136,7 @@
         <v>26</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>26</v>
@@ -1223,11 +1223,9 @@
         <v>26</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>26</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="I9" s="7"/>
     </row>
     <row r="10" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
@@ -1237,7 +1235,7 @@
         <v>4</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>70</v>
@@ -1246,13 +1244,13 @@
         <v>57</v>
       </c>
       <c r="F10" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" s="7" t="s">
         <v>74</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>75</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>26</v>
@@ -1295,7 +1293,7 @@
         <v>2</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>56</v>
@@ -1307,7 +1305,7 @@
         <v>58</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>26</v>
@@ -1324,7 +1322,7 @@
         <v>3</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>56</v>
@@ -1382,7 +1380,7 @@
         <v>5</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>70</v>
@@ -1397,7 +1395,7 @@
         <v>26</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I15" s="7" t="s">
         <v>26</v>
@@ -1440,7 +1438,7 @@
         <v>2</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>56</v>
@@ -1452,7 +1450,7 @@
         <v>58</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H17" s="7" t="s">
         <v>26</v>
@@ -1469,7 +1467,7 @@
         <v>3</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>56</v>
@@ -1481,7 +1479,7 @@
         <v>61</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>26</v>
@@ -1527,16 +1525,16 @@
         <v>5</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>70</v>
       </c>
       <c r="E20" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>86</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>87</v>
       </c>
       <c r="G20" s="7" t="s">
         <v>26</v>

</xml_diff>